<commit_message>
Lift Oscillators done. Testing multistability, in progress.
</commit_message>
<xml_diff>
--- a/apps_results_MAK_REINFORCE/oscillators_lift_3species_6rxns/oscillators_lift_3species_6rxns_MAK_REINFORCE.xlsx
+++ b/apps_results_MAK_REINFORCE/oscillators_lift_3species_6rxns/oscillators_lift_3species_6rxns_MAK_REINFORCE.xlsx
@@ -10,14 +10,14 @@
     <sheet r:id="rId1" sheetId="1" name="Data"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Data'!$A$1:$Y$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Data'!$A$1:$Y$18</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="96">
   <si>
     <t>Timestamp</t>
   </si>
@@ -94,127 +94,217 @@
     <t>t0</t>
   </si>
   <si>
-    <t>2025-11-26 14:21:31</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/d25b2ae6cd20413d85ceacde9e894027</t>
+    <t>2025-11-27 09:52:23</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/ca9718f24bf642c0bae386a86045881b</t>
+  </si>
+  <si>
+    <t>Yes*</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Run was succesful.</t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 5.0, 'entropy_weight_continuous_head': 0.5, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+  </si>
+  <si>
+    <t>0.0001</t>
+  </si>
+  <si>
+    <t>(6, 3, 1, 1280)</t>
+  </si>
+  <si>
+    <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+  </si>
+  <si>
+    <t>{'type': 'lognormal_1D'}</t>
+  </si>
+  <si>
+    <t>{'target_entropy_ratio_to_max': np.float64(0.35679185088982296), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+  </si>
+  <si>
+    <t>[0.4, 0.0, 0.2, 0.4]</t>
+  </si>
+  <si>
+    <t>20.0</t>
+  </si>
+  <si>
+    <t>2025-11-27 16:24:31</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/75d6365eb2fb46e7915c0f99419687be</t>
+  </si>
+  <si>
+    <t>Increased the entropy weight of the structure head. Topological diversity was very high.</t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 10.0, 'entropy_weight_continuous_head': 0.5, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+  </si>
+  <si>
+    <t>2025-11-28 12:06:12</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/5076a726520445789ff4b355a6317b60</t>
+  </si>
+  <si>
+    <t>Successful.</t>
+  </si>
+  <si>
+    <t>2025-12-01 10:06:16</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/de6a4e8fb53b4c44ba8e449d0e51282f</t>
+  </si>
+  <si>
+    <t>run-1. Fast convergence. Topological diversity was high.</t>
+  </si>
+  <si>
+    <t>2025-12-01 15:07:33</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/775c05786f2f4e08a2030cd8ebe0478f</t>
   </si>
   <si>
     <t>Yes/No</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Best samples converged, but the topk average had still a high loss. Got only one topology.</t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
-  </si>
-  <si>
-    <t>0.0001</t>
-  </si>
-  <si>
-    <t>(6, 3, 1, 1280)</t>
-  </si>
-  <si>
-    <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
-  </si>
-  <si>
-    <t>{'type': 'lognormal_1D'}</t>
-  </si>
-  <si>
-    <t>{'target_entropy_ratio_to_max': np.float64(0.35679185088982296), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
-  </si>
-  <si>
-    <t>[0.4, 0.0, 0.2, 0.4]</t>
-  </si>
-  <si>
-    <t>20.0</t>
-  </si>
-  <si>
-    <t>2025-11-26 15:51:57</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/19c9380773ab4bbaac23c032943012ee</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
-    <t>Decreased the global entropy weight significantly. Collapsed.</t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 1e-05, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
-  </si>
-  <si>
-    <t>2025-11-26 16:15:06</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/1519137a59584ee1a501b8c5c84ae60f</t>
-  </si>
-  <si>
-    <t>Increased the global entropy. Didn't help</t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.0001, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
-  </si>
-  <si>
-    <t>2025-11-26 17:23:25</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/cf49e39472a54d7985cdd4d9f8a88f6e</t>
-  </si>
-  <si>
-    <t>Increased the global entropy weight. Also increased the entorpy weight of the structure head. Maybe not enough epochs.</t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 2.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
-  </si>
-  <si>
-    <t>2025-11-26 18:14:07</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/fbf031cbda634e009b417496c7c85308</t>
-  </si>
-  <si>
-    <t>Increased epochs. Got one topology.</t>
-  </si>
-  <si>
-    <t>2025-11-26 21:13:19</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/e0f0e2a39e9143c9856e3e1dbbea7f9c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Increased the entropy weight on the structure head. Better, but very few topologies. </t>
+    <t>run-2. Structure-Entropy weight = 2 x Parameter-Entropy weight. One topology obtained.</t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 0.5, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+  </si>
+  <si>
+    <t>2025-12-01 15:52:35</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/5b6c2246abc64a93bfde8344f29d85c8</t>
+  </si>
+  <si>
+    <t>run-3. Structure-Entropy weight = 4 x Parameter-Entropy weight. One topology obtained.</t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 2.0, 'entropy_weight_continuous_head': 0.5, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+  </si>
+  <si>
+    <t>2025-12-01 16:40:33</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/5c5e5e334f644abaa87c2652ba779598</t>
+  </si>
+  <si>
+    <t xml:space="preserve">run-4. Structure-Entropy weight = 8 x Parameter-Entropy weight. Topology diversity is better. </t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 4.0, 'entropy_weight_continuous_head': 0.5, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+  </si>
+  <si>
+    <t>2025-12-01 18:08:12</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/4a54eb22fb4f4a1faddf3c00e46b2223</t>
+  </si>
+  <si>
+    <t>run-5. Same conditions as previous run. Consistent results.</t>
+  </si>
+  <si>
+    <t>2025-12-02 08:47:41</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/466fd7d9dc104cc683bc463e6443b3c2</t>
+  </si>
+  <si>
+    <t>run-6. Same conditions as previous run. Convergence was slower but more steady.  Diversity was high.</t>
+  </si>
+  <si>
+    <t>2025-12-02 09:26:45</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/6a0dc10994a54ee2a29e4f053975aedc</t>
+  </si>
+  <si>
+    <t>run-7. Set the entropy weights of the heads to [5, 1]. No topological diversity</t>
   </si>
   <si>
     <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 5.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
   </si>
   <si>
-    <t>2025-11-27 07:47:52</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/9bc2bc96f2954e0b9f2f2f6ade065139</t>
-  </si>
-  <si>
-    <t>Decreased the entropy weight on the parameter head. Very few topologies.</t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 5.0, 'entropy_weight_continuous_head': 0.5, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
-  </si>
-  <si>
-    <t>2025-11-27 09:52:23</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/ca9718f24bf642c0bae386a86045881b</t>
-  </si>
-  <si>
-    <t>Increased the risk to 0.95.</t>
-  </si>
-  <si>
-    <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+    <t>2025-12-02 11:25:39</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/f187bccd5ddf435f8967a011bb290a1a</t>
+  </si>
+  <si>
+    <t>run-8. Set the entropy weights of the heads to [10, 1]. No convergence</t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 10.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+  </si>
+  <si>
+    <t>2025-12-02 12:32:04</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/e626bb66008047caa8677c06ec8d73a7</t>
+  </si>
+  <si>
+    <t>run-9. Set the entropy weights of the heads to [1, 0.1]. Good topological diversity</t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 1.0, 'entropy_weight_continuous_head': 0.1, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+  </si>
+  <si>
+    <t>2025-12-02 15:03:55</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/27445fca6ec3481baf970fc5b98d9eed</t>
+  </si>
+  <si>
+    <t>run-10. Same conditions as previous run. Successful but small oscillations.</t>
+  </si>
+  <si>
+    <t>2025-12-02 16:13:38</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/65e379d8e19949ceb71989fc29058e2f</t>
+  </si>
+  <si>
+    <t>run-11. Same conditions as previous run. Succesful but worst topk fluctuated a lot.</t>
+  </si>
+  <si>
+    <t>2025-12-02 17:51:08</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/7b9ae9d929d647d8b2d337220df8ce32</t>
+  </si>
+  <si>
+    <t>run-12. Set the entropy weights of the heads to [7.5, 0.5]. Most successful run so far.</t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 7.5, 'entropy_weight_continuous_head': 0.5, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+  </si>
+  <si>
+    <t>2025-12-03 07:10:34</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/ae02a8b3547c4effab370437ff3c96c0</t>
+  </si>
+  <si>
+    <t>run-13. Same conditions as previous run. Excellent results.</t>
+  </si>
+  <si>
+    <t>2025-12-03 09:22:55</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/oscillators-lift-3species-6rxns-mak-reinforce/a43f04dd528a4ad281ac4378397a74ee</t>
+  </si>
+  <si>
+    <t>run-14. Same conditions as previous run. Excellent results.</t>
   </si>
 </sst>
 </file>
@@ -222,7 +312,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,12 +323,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -270,15 +354,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -589,34 +670,34 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:Y9"/>
+  <dimension ref="A1:Y18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="20.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="11.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="4" width="6.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="119.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="255.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="4" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="7.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="4" width="75.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="5" width="21.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="5" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="4" width="25.005" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="4" width="134.005" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="4" width="21.005" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="4" width="5.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="3" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="3" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="3" width="11.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="3" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="3" width="6.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="3" width="101.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="3" width="255.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="3" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="4" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="3" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="4" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="4" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="4" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="4" width="7.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="3" width="75.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="4" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="4" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="4" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="4" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="4" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="4" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="3" width="25.005" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="3" width="134.005" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="3" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="3" width="5.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -722,7 +803,7 @@
         <v>31</v>
       </c>
       <c r="I2" s="2">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>32</v>
@@ -781,25 +862,25 @@
         <v>39</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>31</v>
       </c>
       <c r="I3" s="2">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>32</v>
@@ -852,31 +933,31 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="G4" s="1" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>31</v>
       </c>
       <c r="I4" s="2">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>32</v>
@@ -929,10 +1010,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>27</v>
@@ -944,16 +1025,16 @@
         <v>28</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>31</v>
       </c>
       <c r="I5" s="2">
-        <v>300</v>
+        <v>700</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>32</v>
@@ -1006,31 +1087,31 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>31</v>
       </c>
       <c r="I6" s="2">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>32</v>
@@ -1089,13 +1170,13 @@
         <v>55</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>28</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>56</v>
@@ -1107,7 +1188,7 @@
         <v>31</v>
       </c>
       <c r="I7" s="2">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>32</v>
@@ -1166,7 +1247,7 @@
         <v>59</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>28</v>
@@ -1184,7 +1265,7 @@
         <v>31</v>
       </c>
       <c r="I8" s="2">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>32</v>
@@ -1235,16 +1316,22 @@
         <v>37</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
+      <c r="C9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>28</v>
+      </c>
       <c r="F9" s="1" t="s">
         <v>64</v>
       </c>
@@ -1254,43 +1341,43 @@
       <c r="H9" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="I9" s="3">
-        <v>500</v>
+      <c r="I9" s="2">
+        <v>400</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K9" s="3">
+      <c r="K9" s="2">
         <v>5</v>
       </c>
-      <c r="L9" s="3">
+      <c r="L9" s="2">
         <v>1024</v>
       </c>
-      <c r="M9" s="3">
+      <c r="M9" s="2">
         <v>10240</v>
       </c>
-      <c r="N9" s="3">
+      <c r="N9" s="2">
         <v>128</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="P9" s="3">
+        <v>33</v>
+      </c>
+      <c r="P9" s="2">
         <v>10</v>
       </c>
-      <c r="Q9" s="3">
+      <c r="Q9" s="2">
         <v>30</v>
       </c>
-      <c r="R9" s="3">
+      <c r="R9" s="2">
         <v>100</v>
       </c>
-      <c r="S9" s="3">
+      <c r="S9" s="2">
         <v>1000</v>
       </c>
-      <c r="T9" s="3">
-        <v>1</v>
-      </c>
-      <c r="U9" s="3">
+      <c r="T9" s="2">
+        <v>1</v>
+      </c>
+      <c r="U9" s="2">
         <v>1</v>
       </c>
       <c r="V9" s="1" t="s">
@@ -1303,6 +1390,699 @@
         <v>36</v>
       </c>
       <c r="Y9" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="2">
+        <v>400</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K10" s="2">
+        <v>5</v>
+      </c>
+      <c r="L10" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M10" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N10" s="2">
+        <v>128</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P10" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>30</v>
+      </c>
+      <c r="R10" s="2">
+        <v>100</v>
+      </c>
+      <c r="S10" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T10" s="2">
+        <v>1</v>
+      </c>
+      <c r="U10" s="2">
+        <v>1</v>
+      </c>
+      <c r="V10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="X10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y10" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="2">
+        <v>400</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K11" s="2">
+        <v>5</v>
+      </c>
+      <c r="L11" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M11" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N11" s="2">
+        <v>128</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P11" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>30</v>
+      </c>
+      <c r="R11" s="2">
+        <v>100</v>
+      </c>
+      <c r="S11" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T11" s="2">
+        <v>1</v>
+      </c>
+      <c r="U11" s="2">
+        <v>1</v>
+      </c>
+      <c r="V11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="X11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y11" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I12" s="2">
+        <v>400</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K12" s="2">
+        <v>5</v>
+      </c>
+      <c r="L12" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M12" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N12" s="2">
+        <v>128</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P12" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>30</v>
+      </c>
+      <c r="R12" s="2">
+        <v>100</v>
+      </c>
+      <c r="S12" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T12" s="2">
+        <v>1</v>
+      </c>
+      <c r="U12" s="2">
+        <v>1</v>
+      </c>
+      <c r="V12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W12" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="X12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y12" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I13" s="2">
+        <v>400</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K13" s="2">
+        <v>5</v>
+      </c>
+      <c r="L13" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M13" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N13" s="2">
+        <v>128</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P13" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>30</v>
+      </c>
+      <c r="R13" s="2">
+        <v>100</v>
+      </c>
+      <c r="S13" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T13" s="2">
+        <v>1</v>
+      </c>
+      <c r="U13" s="2">
+        <v>1</v>
+      </c>
+      <c r="V13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="X13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y13" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="2">
+        <v>700</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K14" s="2">
+        <v>5</v>
+      </c>
+      <c r="L14" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M14" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N14" s="2">
+        <v>128</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P14" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>30</v>
+      </c>
+      <c r="R14" s="2">
+        <v>100</v>
+      </c>
+      <c r="S14" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T14" s="2">
+        <v>1</v>
+      </c>
+      <c r="U14" s="2">
+        <v>1</v>
+      </c>
+      <c r="V14" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W14" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="X14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y14" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="A15" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I15" s="2">
+        <v>700</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K15" s="2">
+        <v>5</v>
+      </c>
+      <c r="L15" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M15" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N15" s="2">
+        <v>128</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P15" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>30</v>
+      </c>
+      <c r="R15" s="2">
+        <v>100</v>
+      </c>
+      <c r="S15" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T15" s="2">
+        <v>1</v>
+      </c>
+      <c r="U15" s="2">
+        <v>1</v>
+      </c>
+      <c r="V15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W15" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="X15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y15" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I16" s="2">
+        <v>700</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K16" s="2">
+        <v>5</v>
+      </c>
+      <c r="L16" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M16" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N16" s="2">
+        <v>128</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P16" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>30</v>
+      </c>
+      <c r="R16" s="2">
+        <v>100</v>
+      </c>
+      <c r="S16" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T16" s="2">
+        <v>1</v>
+      </c>
+      <c r="U16" s="2">
+        <v>1</v>
+      </c>
+      <c r="V16" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="X16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y16" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="A17" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I17" s="2">
+        <v>700</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K17" s="2">
+        <v>5</v>
+      </c>
+      <c r="L17" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M17" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N17" s="2">
+        <v>128</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P17" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>30</v>
+      </c>
+      <c r="R17" s="2">
+        <v>100</v>
+      </c>
+      <c r="S17" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T17" s="2">
+        <v>1</v>
+      </c>
+      <c r="U17" s="2">
+        <v>1</v>
+      </c>
+      <c r="V17" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W17" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="X17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y17" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+      <c r="A18" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I18" s="2">
+        <v>700</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K18" s="2">
+        <v>5</v>
+      </c>
+      <c r="L18" s="2">
+        <v>1024</v>
+      </c>
+      <c r="M18" s="2">
+        <v>10240</v>
+      </c>
+      <c r="N18" s="2">
+        <v>128</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P18" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>30</v>
+      </c>
+      <c r="R18" s="2">
+        <v>100</v>
+      </c>
+      <c r="S18" s="2">
+        <v>1000</v>
+      </c>
+      <c r="T18" s="2">
+        <v>1</v>
+      </c>
+      <c r="U18" s="2">
+        <v>1</v>
+      </c>
+      <c r="V18" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="X18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y18" s="1" t="s">
         <v>37</v>
       </c>
     </row>

</xml_diff>